<commit_message>
Añadimos activos en euros
He añadido un ETF en euros a la cartera. Ha sido necesario hacer algunos cambios porque antes asumía que todo estaba en la misma divisa.
</commit_message>
<xml_diff>
--- a/Libro_inversiones.xlsx
+++ b/Libro_inversiones.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Cuentas\Inversiones\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Cuentas\Seguimiento_cartera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090475EA-D151-4C30-8E8D-5BE41763212E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C45DFE5-D83C-4B76-B0C5-6B5F0BE83297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1139A198-E72E-464B-B201-8BF5D45D4D37}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="23">
   <si>
     <t>Activo</t>
   </si>
@@ -90,15 +90,22 @@
   </si>
   <si>
     <t>Aportación</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>S500.MI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0.000000_-;\-* #,##0.000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.000000_-;\-* #,##0.000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.00000000_-;\-* #,##0.00000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -137,20 +144,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
-      <numFmt numFmtId="168" formatCode="_-* #,##0.000000_-;\-* #,##0.000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="169" formatCode="_-* #,##0.00000000_-;\-* #,##0.00000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.000000_-;\-* #,##0.000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
@@ -172,13 +184,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}" name="Table2" displayName="Table2" ref="A1:F7" totalsRowShown="0">
-  <autoFilter ref="A1:F7" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}" name="Table2" displayName="Table2" ref="A1:F8" totalsRowShown="0">
+  <autoFilter ref="A1:F8" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{7ACE7E66-3686-44B0-B231-8C83869515C6}" name="Activo"/>
-    <tableColumn id="2" xr3:uid="{94864417-15F3-4F84-A992-4D4414E20F6A}" name="Fecha" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{94864417-15F3-4F84-A992-4D4414E20F6A}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{8354A1CC-EF2A-4225-BAC8-5C2695D9A394}" name="Orden"/>
-    <tableColumn id="4" xr3:uid="{7F9F7DD8-9903-4B4D-9EC3-05C05949EE90}" name="Numero_acciones"/>
+    <tableColumn id="4" xr3:uid="{7F9F7DD8-9903-4B4D-9EC3-05C05949EE90}" name="Numero_acciones" dataDxfId="0" dataCellStyle="Comma"/>
     <tableColumn id="5" xr3:uid="{6F579681-2E5F-4386-B799-C0B02978B701}" name="Precio_ejecutado" dataCellStyle="Comma"/>
     <tableColumn id="6" xr3:uid="{134F58B4-8F40-4F5E-A117-6BD376E02A72}" name="Currency"/>
   </tableColumns>
@@ -187,14 +199,14 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}" name="Table3" displayName="Table3" ref="A1:E5" totalsRowShown="0">
-  <autoFilter ref="A1:E5" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}" name="Table3" displayName="Table3" ref="A1:E6" totalsRowShown="0">
+  <autoFilter ref="A1:E6" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{ACF46425-D07B-40C6-814D-C1294D2F317A}" name="Fecha" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{ACF46425-D07B-40C6-814D-C1294D2F317A}" name="Fecha" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{C9D64245-6F89-4E17-B03B-18349867EB64}" name="Tipo"/>
     <tableColumn id="3" xr3:uid="{AE3235F4-616A-423A-A187-7B65E09D4386}" name="Importe"/>
     <tableColumn id="4" xr3:uid="{AB17CC25-F7B9-4B8C-8AF2-4AA81F840A42}" name="Currency"/>
-    <tableColumn id="5" xr3:uid="{8969ACFC-73CE-45E0-8B09-26B0C3F31FF4}" name="Tipo_cambio_EUR" dataDxfId="0" dataCellStyle="Comma"/>
+    <tableColumn id="5" xr3:uid="{8969ACFC-73CE-45E0-8B09-26B0C3F31FF4}" name="Tipo_cambio_EUR" dataDxfId="1" dataCellStyle="Comma"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -508,12 +520,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA5B4226-CEDB-4702-B055-D0664E4C0BEE}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="4" max="4" width="19" style="6" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -526,7 +539,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -546,7 +559,7 @@
       <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="6">
         <v>0.22963995000000001</v>
       </c>
       <c r="E2" s="2">
@@ -566,7 +579,7 @@
       <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="6">
         <v>0.12937694</v>
       </c>
       <c r="E3" s="2">
@@ -586,7 +599,7 @@
       <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="6">
         <v>0.14394012</v>
       </c>
       <c r="E4" s="2">
@@ -606,7 +619,7 @@
       <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="6">
         <v>0.14394012</v>
       </c>
       <c r="E5" s="2">
@@ -626,7 +639,7 @@
       <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="6">
         <v>0.20754269</v>
       </c>
       <c r="E6" s="2">
@@ -646,7 +659,7 @@
       <c r="C7" t="s">
         <v>9</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="6">
         <v>0.36755086999999997</v>
       </c>
       <c r="E7" s="2">
@@ -656,6 +669,27 @@
         <v>11</v>
       </c>
       <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46175</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="6">
+        <v>0.26326874473462514</v>
+      </c>
+      <c r="E8" s="2">
+        <v>189.92</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -667,7 +701,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85C821D-EDAB-4EB5-8E9C-F5D6DA5F796D}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -761,6 +795,23 @@
         <v>0.86366666666666669</v>
       </c>
     </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>46175</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Correcciones mínimas y nueva página de Histórico
He implementado algunos cambios mínimos de formato generales. Se añade una nueva página de histórico. El objetivo de esta página es dar información sobre el desempeño histórico de la cartera, con datos agregados mensualmente y anualmente.
</commit_message>
<xml_diff>
--- a/Libro_inversiones.xlsx
+++ b/Libro_inversiones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Cuentas\Seguimiento_cartera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52CEC811-BD8C-41A4-BCE6-E765C1CBBF73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8308AB-ACFC-4B84-B1EF-4A3B22CC3301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1139A198-E72E-464B-B201-8BF5D45D4D37}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1139A198-E72E-464B-B201-8BF5D45D4D37}"/>
   </bookViews>
   <sheets>
     <sheet name="Operaciones" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="57">
   <si>
     <t>Activo</t>
   </si>
@@ -286,8 +286,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}" name="Table2" displayName="Table2" ref="A1:G10" totalsRowShown="0">
-  <autoFilter ref="A1:G10" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}" name="Table2" displayName="Table2" ref="A1:G12" totalsRowShown="0">
+  <autoFilter ref="A1:G12" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{7ACE7E66-3686-44B0-B231-8C83869515C6}" name="Activo"/>
     <tableColumn id="2" xr3:uid="{94864417-15F3-4F84-A992-4D4414E20F6A}" name="Fecha" dataDxfId="3"/>
@@ -302,8 +302,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}" name="Table3" displayName="Table3" ref="A1:F9" totalsRowShown="0">
-  <autoFilter ref="A1:F9" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}" name="Table3" displayName="Table3" ref="A1:F12" totalsRowShown="0">
+  <autoFilter ref="A1:F12" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{ACF46425-D07B-40C6-814D-C1294D2F317A}" name="Fecha" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{C9D64245-6F89-4E17-B03B-18349867EB64}" name="Tipo"/>
@@ -626,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA5B4226-CEDB-4702-B055-D0664E4C0BEE}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
@@ -869,6 +869,52 @@
         <v>25</v>
       </c>
     </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46175</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0.25992900000000002</v>
+      </c>
+      <c r="E11" s="2">
+        <v>192.36022144508692</v>
+      </c>
+      <c r="F11" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1">
+        <v>46175</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="6">
+        <v>3.3582000000000001E-2</v>
+      </c>
+      <c r="E12" s="2">
+        <v>192.36495741766421</v>
+      </c>
+      <c r="F12" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -879,7 +925,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85C821D-EDAB-4EB5-8E9C-F5D6DA5F796D}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -1064,6 +1110,63 @@
       </c>
       <c r="F9" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>46199</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10">
+        <v>0.2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>50</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12">
+        <v>6.46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrección de errores y mejora de la investigación
</commit_message>
<xml_diff>
--- a/Libro_inversiones.xlsx
+++ b/Libro_inversiones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Cuentas\Seguimiento_cartera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8308AB-ACFC-4B84-B1EF-4A3B22CC3301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BA676A-D3C4-40C9-BA79-646578D57451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1139A198-E72E-464B-B201-8BF5D45D4D37}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="64">
   <si>
     <t>Activo</t>
   </si>
@@ -198,16 +198,38 @@
   </si>
   <si>
     <t>Dividendo</t>
+  </si>
+  <si>
+    <t>AI3A.F</t>
+  </si>
+  <si>
+    <t>Amadeus</t>
+  </si>
+  <si>
+    <t>Amundi MSCI World Ex USA</t>
+  </si>
+  <si>
+    <t>WEXE.DE</t>
+  </si>
+  <si>
+    <t>Ardtur European Focus</t>
+  </si>
+  <si>
+    <t>0P0001OFHN.F</t>
+  </si>
+  <si>
+    <t>^STOXX50</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.000000_-;\-* #,##0.000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00000000_-;\-* #,##0.00000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="172" formatCode="_-* #,##0.0000_-;\-* #,##0.0000_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -246,7 +268,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -254,6 +276,7 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -286,8 +309,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}" name="Table2" displayName="Table2" ref="A1:G12" totalsRowShown="0">
-  <autoFilter ref="A1:G12" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}" name="Table2" displayName="Table2" ref="A1:G16" totalsRowShown="0">
+  <autoFilter ref="A1:G16" xr:uid="{4FBD09E8-CC38-4211-8F45-37F0AD8CFE23}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{7ACE7E66-3686-44B0-B231-8C83869515C6}" name="Activo"/>
     <tableColumn id="2" xr3:uid="{94864417-15F3-4F84-A992-4D4414E20F6A}" name="Fecha" dataDxfId="3"/>
@@ -302,8 +325,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}" name="Table3" displayName="Table3" ref="A1:F12" totalsRowShown="0">
-  <autoFilter ref="A1:F12" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}" name="Table3" displayName="Table3" ref="A1:F17" totalsRowShown="0">
+  <autoFilter ref="A1:F17" xr:uid="{24C0F87E-F257-4DAE-9A8A-E834BA433B65}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{ACF46425-D07B-40C6-814D-C1294D2F317A}" name="Fecha" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{C9D64245-6F89-4E17-B03B-18349867EB64}" name="Tipo"/>
@@ -317,8 +340,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65789449-B85E-45C7-A107-E4F6D80369A5}" name="Table1" displayName="Table1" ref="A1:D17" totalsRowShown="0">
-  <autoFilter ref="A1:D17" xr:uid="{65789449-B85E-45C7-A107-E4F6D80369A5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65789449-B85E-45C7-A107-E4F6D80369A5}" name="Table1" displayName="Table1" ref="A1:D20" totalsRowShown="0">
+  <autoFilter ref="A1:D20" xr:uid="{65789449-B85E-45C7-A107-E4F6D80369A5}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8BDDDF78-B9AC-4AA8-9374-358359336853}" name="Ticker"/>
     <tableColumn id="2" xr3:uid="{DCB0B9C4-1186-4C96-B726-FF3C19CD750F}" name="Nombre"/>
@@ -626,11 +649,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA5B4226-CEDB-4702-B055-D0664E4C0BEE}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" style="6" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" customWidth="1"/>
     <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -913,6 +936,98 @@
       </c>
       <c r="G12" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="1">
+        <v>46230</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0.99449469000000001</v>
+      </c>
+      <c r="E13" s="2">
+        <v>50.860000066968681</v>
+      </c>
+      <c r="F13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="1">
+        <v>46237</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="6">
+        <v>2.9600999999999999E-2</v>
+      </c>
+      <c r="E14" s="2">
+        <v>192.22323570149661</v>
+      </c>
+      <c r="F14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="1">
+        <v>46237</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="6">
+        <v>4.1267740000000002</v>
+      </c>
+      <c r="E15" s="2">
+        <v>12.116001506261307</v>
+      </c>
+      <c r="F15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46247</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="6">
+        <v>2.8894000000000002</v>
+      </c>
+      <c r="E16" s="7">
+        <v>34.609261438360903</v>
+      </c>
+      <c r="F16" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -925,10 +1040,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85C821D-EDAB-4EB5-8E9C-F5D6DA5F796D}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.28515625" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="19" style="3" customWidth="1"/>
@@ -1114,7 +1230,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>46199</v>
+        <v>46204</v>
       </c>
       <c r="B10" t="s">
         <v>56</v>
@@ -1167,6 +1283,103 @@
       </c>
       <c r="F12" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46217</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13">
+        <v>0.68</v>
+      </c>
+      <c r="D13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>46230</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14">
+        <v>50</v>
+      </c>
+      <c r="D14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="3">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15">
+        <v>5.69</v>
+      </c>
+      <c r="D15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>46237</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16">
+        <v>50</v>
+      </c>
+      <c r="D16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>46247</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17">
+        <v>99.99</v>
+      </c>
+      <c r="D17" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1179,11 +1392,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D94661A8-E3EF-4B91-81A4-2C9D976A1BF9}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1255,10 +1469,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
         <v>30</v>
@@ -1266,38 +1480,35 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
-      </c>
-      <c r="D7" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>30</v>
@@ -1308,10 +1519,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>30</v>
@@ -1322,10 +1533,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
         <v>30</v>
@@ -1336,10 +1547,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
         <v>30</v>
@@ -1350,10 +1561,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
         <v>30</v>
@@ -1364,10 +1575,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
         <v>30</v>
@@ -1378,10 +1589,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
         <v>30</v>
@@ -1392,10 +1603,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
         <v>30</v>
@@ -1406,16 +1617,58 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
         <v>30</v>
       </c>
       <c r="D17" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>